<commit_message>
Update comparison tabs to Jun vs Jul; quarterly data through Q1'27 + July'26
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/CV_Comparison.xlsx
+++ b/CV_Comparison.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Deepanshi Ahuja\Desktop\Marketing_Performance_dashboard\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E556EAAD-1A97-4AE0-8824-5EA78C2F3698}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{85AB68F4-FE03-4E9C-B248-BC28C6664D9F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" xr2:uid="{2A06160F-D6CF-40AF-81FB-3972BB152925}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="122" uniqueCount="41">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="129" uniqueCount="42">
   <si>
     <t>Spends</t>
   </si>
@@ -162,6 +162,9 @@
   </si>
   <si>
     <t>Jul'26</t>
+  </si>
+  <si>
+    <t>Aug'26</t>
   </si>
 </sst>
 </file>
@@ -538,54 +541,61 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{36EECC82-B786-4F88-BF54-40C3395F4A7F}">
-  <dimension ref="A1:AE30"/>
+  <dimension ref="A1:AL30"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="1" spans="1:31" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:38" x14ac:dyDescent="0.35">
       <c r="D1" s="3" t="s">
         <v>0</v>
       </c>
       <c r="E1" s="3"/>
       <c r="F1" s="3"/>
       <c r="G1" s="3"/>
-      <c r="H1" s="3" t="s">
-        <v>1</v>
-      </c>
-      <c r="I1" s="3"/>
+      <c r="H1" s="3"/>
+      <c r="I1" s="3" t="s">
+        <v>1</v>
+      </c>
       <c r="J1" s="3"/>
       <c r="K1" s="3"/>
-      <c r="L1" s="3" t="s">
+      <c r="L1" s="3"/>
+      <c r="M1" s="3"/>
+      <c r="N1" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="M1" s="3"/>
-      <c r="N1" s="3"/>
       <c r="O1" s="3"/>
-      <c r="P1" s="3" t="s">
-        <v>3</v>
-      </c>
+      <c r="P1" s="3"/>
       <c r="Q1" s="3"/>
       <c r="R1" s="3"/>
-      <c r="S1" s="3"/>
-      <c r="T1" s="3" t="s">
-        <v>4</v>
-      </c>
+      <c r="S1" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="T1" s="3"/>
       <c r="U1" s="3"/>
       <c r="V1" s="3"/>
       <c r="W1" s="3"/>
       <c r="X1" s="3" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="Y1" s="3"/>
       <c r="Z1" s="3"/>
       <c r="AA1" s="3"/>
-      <c r="AB1" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="AC1" s="3"/>
+      <c r="AB1" s="3"/>
+      <c r="AC1" s="3" t="s">
+        <v>5</v>
+      </c>
       <c r="AD1" s="3"/>
       <c r="AE1" s="3"/>
+      <c r="AF1" s="3"/>
+      <c r="AG1" s="3"/>
+      <c r="AH1" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="AI1" s="3"/>
+      <c r="AJ1" s="3"/>
+      <c r="AK1" s="3"/>
+      <c r="AL1" s="3"/>
     </row>
-    <row r="2" spans="1:31" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:38" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>7</v>
       </c>
@@ -608,52 +618,52 @@
         <v>40</v>
       </c>
       <c r="H2" t="s">
+        <v>41</v>
+      </c>
+      <c r="I2" t="s">
         <v>10</v>
       </c>
-      <c r="I2" t="s">
+      <c r="J2" t="s">
         <v>11</v>
       </c>
-      <c r="J2" t="s">
+      <c r="K2" t="s">
         <v>12</v>
       </c>
-      <c r="K2" t="s">
+      <c r="L2" t="s">
         <v>40</v>
       </c>
-      <c r="L2" t="s">
+      <c r="M2" t="s">
+        <v>41</v>
+      </c>
+      <c r="N2" t="s">
         <v>10</v>
       </c>
-      <c r="M2" t="s">
+      <c r="O2" t="s">
         <v>11</v>
       </c>
-      <c r="N2" t="s">
+      <c r="P2" t="s">
         <v>12</v>
       </c>
-      <c r="O2" t="s">
+      <c r="Q2" t="s">
         <v>40</v>
       </c>
-      <c r="P2" t="s">
+      <c r="R2" t="s">
+        <v>41</v>
+      </c>
+      <c r="S2" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="Q2" t="s">
+      <c r="T2" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="R2" t="s">
+      <c r="U2" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="S2" s="1" t="s">
+      <c r="V2" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="T2" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="U2" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="V2" s="2" t="s">
-        <v>12</v>
-      </c>
       <c r="W2" s="2" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="X2" s="2" t="s">
         <v>10</v>
@@ -668,19 +678,40 @@
         <v>40</v>
       </c>
       <c r="AB2" t="s">
+        <v>41</v>
+      </c>
+      <c r="AC2" t="s">
         <v>10</v>
       </c>
-      <c r="AC2" t="s">
+      <c r="AD2" t="s">
         <v>11</v>
       </c>
-      <c r="AD2" t="s">
+      <c r="AE2" t="s">
         <v>12</v>
       </c>
-      <c r="AE2" t="s">
+      <c r="AF2" t="s">
         <v>40</v>
       </c>
+      <c r="AG2" t="s">
+        <v>41</v>
+      </c>
+      <c r="AH2" t="s">
+        <v>10</v>
+      </c>
+      <c r="AI2" t="s">
+        <v>11</v>
+      </c>
+      <c r="AJ2" t="s">
+        <v>12</v>
+      </c>
+      <c r="AK2" t="s">
+        <v>40</v>
+      </c>
+      <c r="AL2" t="s">
+        <v>41</v>
+      </c>
     </row>
-    <row r="3" spans="1:31" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:38" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>13</v>
       </c>
@@ -700,82 +731,103 @@
         <v>42267</v>
       </c>
       <c r="G3">
-        <v>5525</v>
+        <v>37710</v>
       </c>
       <c r="H3">
+        <v>3725</v>
+      </c>
+      <c r="I3">
         <v>1621</v>
       </c>
-      <c r="I3">
+      <c r="J3">
         <v>1074</v>
       </c>
-      <c r="J3">
+      <c r="K3">
         <v>1203</v>
       </c>
-      <c r="K3">
-        <v>179</v>
-      </c>
       <c r="L3">
+        <v>1036</v>
+      </c>
+      <c r="M3">
+        <v>89</v>
+      </c>
+      <c r="N3">
         <v>27</v>
       </c>
-      <c r="M3">
+      <c r="O3">
         <v>19</v>
       </c>
-      <c r="N3">
+      <c r="P3">
         <v>35</v>
       </c>
-      <c r="O3">
-        <v>31</v>
-      </c>
-      <c r="P3">
+      <c r="Q3">
+        <v>36</v>
+      </c>
+      <c r="R3">
+        <v>42</v>
+      </c>
+      <c r="S3" s="1">
         <v>639</v>
       </c>
-      <c r="Q3">
+      <c r="T3" s="1">
         <v>1500</v>
       </c>
-      <c r="R3">
+      <c r="U3" s="1">
         <v>2230</v>
       </c>
-      <c r="S3" s="1">
-        <v>386</v>
-      </c>
-      <c r="T3" s="1">
+      <c r="V3" s="2">
+        <v>2102</v>
+      </c>
+      <c r="W3" s="2">
+        <v>0</v>
+      </c>
+      <c r="X3" s="2">
         <v>68</v>
       </c>
-      <c r="U3" s="1">
+      <c r="Y3" s="1">
         <v>14</v>
       </c>
-      <c r="V3" s="2">
+      <c r="Z3" s="1">
         <v>19</v>
       </c>
-      <c r="W3" s="2">
-        <v>14</v>
-      </c>
-      <c r="X3" s="2">
+      <c r="AA3" s="1">
+        <v>18</v>
+      </c>
+      <c r="AB3" s="2">
+        <v>0</v>
+      </c>
+      <c r="AC3" s="2">
         <v>0.77349999999999997</v>
       </c>
-      <c r="Y3" s="1">
+      <c r="AD3" s="2">
         <v>0.95399999999999996</v>
       </c>
-      <c r="Z3" s="1">
+      <c r="AE3" s="2">
         <v>0.93679999999999997</v>
       </c>
-      <c r="AA3" s="1">
-        <v>0</v>
-      </c>
-      <c r="AB3" s="2">
-        <v>1</v>
-      </c>
-      <c r="AC3" s="2">
-        <v>1</v>
-      </c>
-      <c r="AD3" s="2">
-        <v>1</v>
-      </c>
-      <c r="AE3" s="2">
+      <c r="AF3" s="1">
+        <v>0.94020000000000004</v>
+      </c>
+      <c r="AG3" s="1">
+        <v>0</v>
+      </c>
+      <c r="AH3" s="2">
+        <v>1</v>
+      </c>
+      <c r="AI3" s="2">
+        <v>1</v>
+      </c>
+      <c r="AJ3" s="2">
+        <v>1</v>
+      </c>
+      <c r="AK3" s="2">
+        <v>1</v>
+      </c>
+      <c r="AL3" s="2">
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:31" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:38" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>13</v>
       </c>
@@ -795,82 +847,103 @@
         <v>49956</v>
       </c>
       <c r="G4">
-        <v>6133</v>
+        <v>37637</v>
       </c>
       <c r="H4">
+        <v>3836</v>
+      </c>
+      <c r="I4">
         <v>600</v>
       </c>
-      <c r="I4">
+      <c r="J4">
         <v>857</v>
       </c>
-      <c r="J4">
+      <c r="K4">
         <v>1227</v>
       </c>
-      <c r="K4">
-        <v>187</v>
-      </c>
       <c r="L4">
+        <v>1084</v>
+      </c>
+      <c r="M4">
+        <v>111</v>
+      </c>
+      <c r="N4">
         <v>24</v>
       </c>
-      <c r="M4">
+      <c r="O4">
         <v>25</v>
       </c>
-      <c r="N4">
+      <c r="P4">
         <v>41</v>
       </c>
-      <c r="O4">
-        <v>33</v>
-      </c>
-      <c r="P4">
+      <c r="Q4">
+        <v>35</v>
+      </c>
+      <c r="R4">
+        <v>35</v>
+      </c>
+      <c r="S4" s="1">
         <v>517</v>
       </c>
-      <c r="Q4">
+      <c r="T4" s="1">
         <v>1504</v>
       </c>
-      <c r="R4">
+      <c r="U4" s="1">
         <v>2324</v>
       </c>
-      <c r="S4" s="1">
-        <v>356</v>
-      </c>
-      <c r="T4" s="1">
+      <c r="V4" s="2">
+        <v>2244</v>
+      </c>
+      <c r="W4" s="2">
+        <v>0</v>
+      </c>
+      <c r="X4" s="2">
         <v>28</v>
       </c>
-      <c r="U4" s="1">
+      <c r="Y4" s="1">
         <v>14</v>
       </c>
-      <c r="V4" s="2">
+      <c r="Z4" s="1">
         <v>21</v>
       </c>
-      <c r="W4" s="2">
+      <c r="AA4" s="1">
         <v>17</v>
       </c>
-      <c r="X4" s="2">
+      <c r="AB4" s="2">
+        <v>0</v>
+      </c>
+      <c r="AC4" s="2">
         <v>0.90659999999999996</v>
       </c>
-      <c r="Y4" s="1">
+      <c r="AD4" s="2">
         <v>0.95269999999999999</v>
       </c>
-      <c r="Z4" s="1">
+      <c r="AE4" s="2">
         <v>0.92830000000000001</v>
       </c>
-      <c r="AA4" s="1">
-        <v>0</v>
-      </c>
-      <c r="AB4" s="2">
-        <v>1</v>
-      </c>
-      <c r="AC4" s="2">
-        <v>1</v>
-      </c>
-      <c r="AD4" s="2">
-        <v>1</v>
-      </c>
-      <c r="AE4" s="2">
+      <c r="AF4" s="1">
+        <v>0.94410000000000005</v>
+      </c>
+      <c r="AG4" s="1">
+        <v>0</v>
+      </c>
+      <c r="AH4" s="2">
+        <v>1</v>
+      </c>
+      <c r="AI4" s="2">
+        <v>1</v>
+      </c>
+      <c r="AJ4" s="2">
+        <v>1</v>
+      </c>
+      <c r="AK4" s="2">
+        <v>1</v>
+      </c>
+      <c r="AL4" s="2">
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:31" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:38" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>17</v>
       </c>
@@ -893,11 +966,11 @@
         <v>0</v>
       </c>
       <c r="H5">
+        <v>0</v>
+      </c>
+      <c r="I5">
         <v>171</v>
       </c>
-      <c r="I5">
-        <v>0</v>
-      </c>
       <c r="J5">
         <v>0</v>
       </c>
@@ -905,67 +978,88 @@
         <v>0</v>
       </c>
       <c r="L5">
+        <v>0</v>
+      </c>
+      <c r="M5">
+        <v>0</v>
+      </c>
+      <c r="N5">
         <v>8</v>
       </c>
-      <c r="M5">
-        <v>0</v>
-      </c>
-      <c r="N5">
-        <v>0</v>
-      </c>
       <c r="O5">
         <v>0</v>
       </c>
       <c r="P5">
+        <v>0</v>
+      </c>
+      <c r="Q5">
+        <v>0</v>
+      </c>
+      <c r="R5">
+        <v>0</v>
+      </c>
+      <c r="S5" s="1">
         <v>122</v>
       </c>
-      <c r="Q5">
-        <v>0</v>
-      </c>
-      <c r="R5">
-        <v>0</v>
-      </c>
-      <c r="S5" s="1">
-        <v>0</v>
-      </c>
       <c r="T5" s="1">
+        <v>0</v>
+      </c>
+      <c r="U5" s="1">
+        <v>0</v>
+      </c>
+      <c r="V5" s="2">
+        <v>0</v>
+      </c>
+      <c r="W5" s="2">
+        <v>0</v>
+      </c>
+      <c r="X5" s="2">
         <v>11</v>
       </c>
-      <c r="U5" s="1">
-        <v>0</v>
-      </c>
-      <c r="V5" s="2">
-        <v>0</v>
-      </c>
-      <c r="W5" s="2">
-        <v>0</v>
-      </c>
-      <c r="X5" s="2">
+      <c r="Y5" s="1">
+        <v>0</v>
+      </c>
+      <c r="Z5" s="1">
+        <v>0</v>
+      </c>
+      <c r="AA5" s="1">
+        <v>0</v>
+      </c>
+      <c r="AB5" s="2">
+        <v>0</v>
+      </c>
+      <c r="AC5" s="2">
         <v>0.84940000000000004</v>
       </c>
-      <c r="Y5" s="1">
-        <v>0</v>
-      </c>
-      <c r="Z5" s="1">
-        <v>0</v>
-      </c>
-      <c r="AA5" s="1">
-        <v>0</v>
-      </c>
-      <c r="AB5" s="2">
+      <c r="AD5" s="2">
+        <v>0</v>
+      </c>
+      <c r="AE5" s="2">
+        <v>0</v>
+      </c>
+      <c r="AF5" s="1">
+        <v>0</v>
+      </c>
+      <c r="AG5" s="1">
+        <v>0</v>
+      </c>
+      <c r="AH5" s="2">
         <v>0.25</v>
       </c>
-      <c r="AC5" s="2">
+      <c r="AI5" s="2">
         <v>0.25</v>
       </c>
-      <c r="AD5" s="2">
+      <c r="AJ5" s="2">
         <v>0.25</v>
       </c>
-      <c r="AE5" s="2">
+      <c r="AK5" s="2">
         <v>0.25</v>
       </c>
+      <c r="AL5" s="2">
+        <v>0.25</v>
+      </c>
     </row>
-    <row r="6" spans="1:31" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:38" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>19</v>
       </c>
@@ -985,82 +1079,103 @@
         <v>2044</v>
       </c>
       <c r="G6">
-        <v>2992</v>
+        <v>5164</v>
       </c>
       <c r="H6">
+        <v>0</v>
+      </c>
+      <c r="I6">
         <v>649</v>
       </c>
-      <c r="I6">
+      <c r="J6">
         <v>1195</v>
       </c>
-      <c r="J6">
+      <c r="K6">
         <v>92</v>
       </c>
-      <c r="K6">
-        <v>23</v>
-      </c>
       <c r="L6">
+        <v>58</v>
+      </c>
+      <c r="M6">
+        <v>0</v>
+      </c>
+      <c r="N6">
         <v>24</v>
       </c>
-      <c r="M6">
+      <c r="O6">
         <v>34</v>
       </c>
-      <c r="N6">
+      <c r="P6">
         <v>22</v>
       </c>
-      <c r="O6">
-        <v>130</v>
-      </c>
-      <c r="P6">
+      <c r="Q6">
+        <v>89</v>
+      </c>
+      <c r="R6">
+        <v>0</v>
+      </c>
+      <c r="S6" s="1">
         <v>426</v>
       </c>
-      <c r="Q6">
+      <c r="T6" s="1">
         <v>820</v>
       </c>
-      <c r="R6">
+      <c r="U6" s="1">
         <v>15</v>
       </c>
-      <c r="S6" s="1">
-        <v>24</v>
-      </c>
-      <c r="T6" s="1">
+      <c r="V6" s="2">
+        <v>54</v>
+      </c>
+      <c r="W6" s="2">
+        <v>0</v>
+      </c>
+      <c r="X6" s="2">
         <v>36</v>
       </c>
-      <c r="U6" s="1">
+      <c r="Y6" s="1">
         <v>50</v>
       </c>
-      <c r="V6" s="2">
+      <c r="Z6" s="1">
         <v>136</v>
       </c>
-      <c r="W6" s="2">
-        <v>125</v>
-      </c>
-      <c r="X6" s="2">
+      <c r="AA6" s="1">
+        <v>96</v>
+      </c>
+      <c r="AB6" s="2">
+        <v>0</v>
+      </c>
+      <c r="AC6" s="2">
         <v>0.33400000000000002</v>
       </c>
-      <c r="Y6" s="1">
+      <c r="AD6" s="2">
         <v>0.25769999999999998</v>
       </c>
-      <c r="Z6" s="1">
+      <c r="AE6" s="2">
         <v>-1.0189999999999999</v>
       </c>
-      <c r="AA6" s="1">
-        <v>0</v>
-      </c>
-      <c r="AB6" s="2">
+      <c r="AF6" s="1">
+        <v>-1.0246999999999999</v>
+      </c>
+      <c r="AG6" s="1">
+        <v>0</v>
+      </c>
+      <c r="AH6" s="2">
         <v>0.12</v>
       </c>
-      <c r="AC6" s="2">
+      <c r="AI6" s="2">
         <v>0.15</v>
       </c>
-      <c r="AD6" s="2">
+      <c r="AJ6" s="2">
         <v>0.15</v>
       </c>
-      <c r="AE6" s="2">
+      <c r="AK6" s="2">
         <v>0.17</v>
       </c>
+      <c r="AL6" s="2">
+        <v>0.17</v>
+      </c>
     </row>
-    <row r="7" spans="1:31" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:38" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>22</v>
       </c>
@@ -1080,82 +1195,103 @@
         <v>29834</v>
       </c>
       <c r="G7">
-        <v>6922</v>
+        <v>40242</v>
       </c>
       <c r="H7">
+        <v>1802</v>
+      </c>
+      <c r="I7">
         <v>419</v>
       </c>
-      <c r="I7">
+      <c r="J7">
         <v>667</v>
       </c>
-      <c r="J7">
+      <c r="K7">
         <v>646</v>
       </c>
-      <c r="K7">
-        <v>171</v>
-      </c>
       <c r="L7">
+        <v>898</v>
+      </c>
+      <c r="M7">
+        <v>60</v>
+      </c>
+      <c r="N7">
         <v>24</v>
       </c>
-      <c r="M7">
+      <c r="O7">
         <v>35</v>
       </c>
-      <c r="N7">
+      <c r="P7">
         <v>46</v>
       </c>
-      <c r="O7">
-        <v>40</v>
-      </c>
-      <c r="P7">
+      <c r="Q7">
+        <v>45</v>
+      </c>
+      <c r="R7">
+        <v>30</v>
+      </c>
+      <c r="S7" s="1">
         <v>332</v>
       </c>
-      <c r="Q7">
+      <c r="T7" s="1">
         <v>497</v>
       </c>
-      <c r="R7">
+      <c r="U7" s="1">
         <v>516</v>
       </c>
-      <c r="S7" s="1">
-        <v>113</v>
-      </c>
-      <c r="T7" s="1">
+      <c r="V7" s="2">
+        <v>646</v>
+      </c>
+      <c r="W7" s="2">
+        <v>29</v>
+      </c>
+      <c r="X7" s="2">
         <v>31</v>
       </c>
-      <c r="U7" s="1">
+      <c r="Y7" s="1">
         <v>47</v>
       </c>
-      <c r="V7" s="2">
+      <c r="Z7" s="1">
         <v>58</v>
       </c>
-      <c r="W7" s="2">
-        <v>61</v>
-      </c>
-      <c r="X7" s="2">
+      <c r="AA7" s="1">
+        <v>62</v>
+      </c>
+      <c r="AB7" s="2">
+        <v>62</v>
+      </c>
+      <c r="AC7" s="2">
         <v>-9.6799999999999997E-2</v>
       </c>
-      <c r="Y7" s="1">
+      <c r="AD7" s="2">
         <v>0.43290000000000001</v>
       </c>
-      <c r="Z7" s="1">
+      <c r="AE7" s="2">
         <v>0.30170000000000002</v>
       </c>
-      <c r="AA7" s="1">
-        <v>0</v>
-      </c>
-      <c r="AB7" s="2">
+      <c r="AF7" s="1">
+        <v>-0.23599999999999999</v>
+      </c>
+      <c r="AG7" s="1">
+        <v>-0.23280000000000001</v>
+      </c>
+      <c r="AH7" s="2">
         <v>0.08</v>
       </c>
-      <c r="AC7" s="2">
+      <c r="AI7" s="2">
         <v>0.23</v>
       </c>
-      <c r="AD7" s="2">
+      <c r="AJ7" s="2">
         <v>0.23</v>
       </c>
-      <c r="AE7" s="2">
-        <v>0.23</v>
+      <c r="AK7" s="2">
+        <v>0.14000000000000001</v>
+      </c>
+      <c r="AL7" s="2">
+        <v>0.14000000000000001</v>
       </c>
     </row>
-    <row r="8" spans="1:31" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:38" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>22</v>
       </c>
@@ -1175,82 +1311,103 @@
         <v>63885</v>
       </c>
       <c r="G8">
-        <v>6922</v>
+        <v>69016</v>
       </c>
       <c r="H8">
+        <v>6478</v>
+      </c>
+      <c r="I8">
         <v>1423</v>
       </c>
-      <c r="I8">
+      <c r="J8">
         <v>2182</v>
       </c>
-      <c r="J8">
+      <c r="K8">
         <v>3710</v>
       </c>
-      <c r="K8">
-        <v>171</v>
-      </c>
       <c r="L8">
+        <v>898</v>
+      </c>
+      <c r="M8">
+        <v>60</v>
+      </c>
+      <c r="N8">
         <v>16</v>
       </c>
-      <c r="M8">
+      <c r="O8">
         <v>23</v>
       </c>
-      <c r="N8">
+      <c r="P8">
         <v>17</v>
       </c>
-      <c r="O8">
-        <v>40</v>
-      </c>
-      <c r="P8">
+      <c r="Q8">
+        <v>77</v>
+      </c>
+      <c r="R8">
+        <v>108</v>
+      </c>
+      <c r="S8" s="1">
         <v>461</v>
       </c>
-      <c r="Q8">
+      <c r="T8" s="1">
         <v>882</v>
       </c>
-      <c r="R8">
+      <c r="U8" s="1">
         <v>1298</v>
       </c>
-      <c r="S8" s="1">
-        <v>113</v>
-      </c>
-      <c r="T8" s="1">
+      <c r="V8" s="2">
+        <v>646</v>
+      </c>
+      <c r="W8" s="2">
+        <v>29</v>
+      </c>
+      <c r="X8" s="2">
         <v>49</v>
       </c>
-      <c r="U8" s="1">
+      <c r="Y8" s="1">
         <v>58</v>
       </c>
-      <c r="V8" s="2">
+      <c r="Z8" s="1">
         <v>49</v>
       </c>
-      <c r="W8" s="2">
-        <v>61</v>
-      </c>
-      <c r="X8" s="2">
+      <c r="AA8" s="1">
+        <v>107</v>
+      </c>
+      <c r="AB8" s="2">
+        <v>223</v>
+      </c>
+      <c r="AC8" s="2">
         <v>-1.6020000000000001</v>
       </c>
-      <c r="Y8" s="1">
+      <c r="AD8" s="2">
         <v>-0.33450000000000002</v>
       </c>
-      <c r="Z8" s="1">
+      <c r="AE8" s="2">
         <v>-0.51910000000000001</v>
       </c>
-      <c r="AA8" s="1">
-        <v>0</v>
-      </c>
-      <c r="AB8" s="2">
+      <c r="AF8" s="1">
+        <v>-0.23599999999999999</v>
+      </c>
+      <c r="AG8" s="1">
+        <v>-0.23280000000000001</v>
+      </c>
+      <c r="AH8" s="2">
         <v>0.05</v>
       </c>
-      <c r="AC8" s="2">
+      <c r="AI8" s="2">
         <v>0.12</v>
       </c>
-      <c r="AD8" s="2">
+      <c r="AJ8" s="2">
         <v>0.09</v>
       </c>
-      <c r="AE8" s="2">
-        <v>0.23</v>
+      <c r="AK8" s="2">
+        <v>0.14000000000000001</v>
+      </c>
+      <c r="AL8" s="2">
+        <v>0.14000000000000001</v>
       </c>
     </row>
-    <row r="9" spans="1:31" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:38" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>22</v>
       </c>
@@ -1279,11 +1436,11 @@
         <v>0</v>
       </c>
       <c r="J9">
+        <v>0</v>
+      </c>
+      <c r="K9">
         <v>565</v>
       </c>
-      <c r="K9">
-        <v>0</v>
-      </c>
       <c r="L9">
         <v>0</v>
       </c>
@@ -1291,61 +1448,82 @@
         <v>0</v>
       </c>
       <c r="N9">
+        <v>0</v>
+      </c>
+      <c r="O9">
+        <v>0</v>
+      </c>
+      <c r="P9">
         <v>9</v>
       </c>
-      <c r="O9">
-        <v>0</v>
-      </c>
-      <c r="P9">
-        <v>0</v>
-      </c>
       <c r="Q9">
         <v>0</v>
       </c>
       <c r="R9">
+        <v>0</v>
+      </c>
+      <c r="S9" s="1">
+        <v>0</v>
+      </c>
+      <c r="T9" s="1">
+        <v>0</v>
+      </c>
+      <c r="U9" s="1">
         <v>469</v>
       </c>
-      <c r="S9" s="1">
-        <v>0</v>
-      </c>
-      <c r="T9" s="1">
-        <v>0</v>
-      </c>
-      <c r="U9" s="1">
-        <v>0</v>
-      </c>
       <c r="V9" s="2">
+        <v>0</v>
+      </c>
+      <c r="W9" s="2">
+        <v>0</v>
+      </c>
+      <c r="X9" s="2">
+        <v>0</v>
+      </c>
+      <c r="Y9" s="1">
+        <v>0</v>
+      </c>
+      <c r="Z9" s="1">
         <v>10</v>
       </c>
-      <c r="W9" s="2">
-        <v>0</v>
-      </c>
-      <c r="X9" s="2">
-        <v>0</v>
-      </c>
-      <c r="Y9" s="1">
-        <v>0</v>
-      </c>
-      <c r="Z9" s="1">
+      <c r="AA9" s="1">
+        <v>0</v>
+      </c>
+      <c r="AB9" s="2">
+        <v>0</v>
+      </c>
+      <c r="AC9" s="2">
+        <v>0</v>
+      </c>
+      <c r="AD9" s="2">
+        <v>0</v>
+      </c>
+      <c r="AE9" s="2">
         <v>0.90090000000000003</v>
       </c>
-      <c r="AA9" s="1">
-        <v>0</v>
-      </c>
-      <c r="AB9" s="2">
-        <v>0</v>
-      </c>
-      <c r="AC9" s="2">
-        <v>0</v>
-      </c>
-      <c r="AD9" s="2">
+      <c r="AF9" s="1">
+        <v>0</v>
+      </c>
+      <c r="AG9" s="1">
+        <v>0</v>
+      </c>
+      <c r="AH9" s="2">
+        <v>0</v>
+      </c>
+      <c r="AI9" s="2">
+        <v>0</v>
+      </c>
+      <c r="AJ9" s="2">
         <v>0.23</v>
       </c>
-      <c r="AE9" s="2">
+      <c r="AK9" s="2">
         <v>0.23</v>
       </c>
+      <c r="AL9" s="2">
+        <v>0.23</v>
+      </c>
     </row>
-    <row r="10" spans="1:31" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:38" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>22</v>
       </c>
@@ -1374,11 +1552,11 @@
         <v>0</v>
       </c>
       <c r="J10">
+        <v>0</v>
+      </c>
+      <c r="K10">
         <v>865</v>
       </c>
-      <c r="K10">
-        <v>0</v>
-      </c>
       <c r="L10">
         <v>0</v>
       </c>
@@ -1386,61 +1564,82 @@
         <v>0</v>
       </c>
       <c r="N10">
+        <v>0</v>
+      </c>
+      <c r="O10">
+        <v>0</v>
+      </c>
+      <c r="P10">
         <v>22</v>
       </c>
-      <c r="O10">
-        <v>0</v>
-      </c>
-      <c r="P10">
-        <v>0</v>
-      </c>
       <c r="Q10">
         <v>0</v>
       </c>
       <c r="R10">
+        <v>0</v>
+      </c>
+      <c r="S10" s="1">
+        <v>0</v>
+      </c>
+      <c r="T10" s="1">
+        <v>0</v>
+      </c>
+      <c r="U10" s="1">
         <v>1117</v>
       </c>
-      <c r="S10" s="1">
-        <v>0</v>
-      </c>
-      <c r="T10" s="1">
-        <v>0</v>
-      </c>
-      <c r="U10" s="1">
-        <v>0</v>
-      </c>
       <c r="V10" s="2">
+        <v>0</v>
+      </c>
+      <c r="W10" s="2">
+        <v>0</v>
+      </c>
+      <c r="X10" s="2">
+        <v>0</v>
+      </c>
+      <c r="Y10" s="1">
+        <v>0</v>
+      </c>
+      <c r="Z10" s="1">
         <v>17</v>
       </c>
-      <c r="W10" s="2">
-        <v>0</v>
-      </c>
-      <c r="X10" s="2">
-        <v>0</v>
-      </c>
-      <c r="Y10" s="1">
-        <v>0</v>
-      </c>
-      <c r="Z10" s="1">
+      <c r="AA10" s="1">
+        <v>0</v>
+      </c>
+      <c r="AB10" s="2">
+        <v>0</v>
+      </c>
+      <c r="AC10" s="2">
+        <v>0</v>
+      </c>
+      <c r="AD10" s="2">
+        <v>0</v>
+      </c>
+      <c r="AE10" s="2">
         <v>0.61509999999999998</v>
       </c>
-      <c r="AA10" s="1">
-        <v>0</v>
-      </c>
-      <c r="AB10" s="2">
-        <v>0</v>
-      </c>
-      <c r="AC10" s="2">
-        <v>0</v>
-      </c>
-      <c r="AD10" s="2">
+      <c r="AF10" s="1">
+        <v>0</v>
+      </c>
+      <c r="AG10" s="1">
+        <v>0</v>
+      </c>
+      <c r="AH10" s="2">
+        <v>0</v>
+      </c>
+      <c r="AI10" s="2">
+        <v>0</v>
+      </c>
+      <c r="AJ10" s="2">
         <v>0.1</v>
       </c>
-      <c r="AE10" s="2">
+      <c r="AK10" s="2">
         <v>0.23</v>
       </c>
+      <c r="AL10" s="2">
+        <v>0.23</v>
+      </c>
     </row>
-    <row r="11" spans="1:31" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:38" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>22</v>
       </c>
@@ -1460,82 +1659,103 @@
         <v>30871</v>
       </c>
       <c r="G11">
-        <v>7034</v>
+        <v>55253</v>
       </c>
       <c r="H11">
+        <v>275</v>
+      </c>
+      <c r="I11">
         <v>571</v>
       </c>
-      <c r="I11">
+      <c r="J11">
         <v>265</v>
       </c>
-      <c r="J11">
+      <c r="K11">
         <v>711</v>
       </c>
-      <c r="K11">
-        <v>170</v>
-      </c>
       <c r="L11">
+        <v>1130</v>
+      </c>
+      <c r="M11">
+        <v>12</v>
+      </c>
+      <c r="N11">
         <v>52</v>
       </c>
-      <c r="M11">
+      <c r="O11">
         <v>47</v>
       </c>
-      <c r="N11">
+      <c r="P11">
         <v>43</v>
       </c>
-      <c r="O11">
-        <v>41</v>
-      </c>
-      <c r="P11">
+      <c r="Q11">
+        <v>49</v>
+      </c>
+      <c r="R11">
+        <v>23</v>
+      </c>
+      <c r="S11" s="1">
         <v>422</v>
       </c>
-      <c r="Q11">
+      <c r="T11" s="1">
         <v>186</v>
       </c>
-      <c r="R11">
+      <c r="U11" s="1">
         <v>536</v>
       </c>
-      <c r="S11" s="1">
-        <v>110</v>
-      </c>
-      <c r="T11" s="1">
+      <c r="V11" s="2">
+        <v>714</v>
+      </c>
+      <c r="W11" s="2">
+        <v>6</v>
+      </c>
+      <c r="X11" s="2">
         <v>70</v>
       </c>
-      <c r="U11" s="1">
+      <c r="Y11" s="1">
         <v>67</v>
       </c>
-      <c r="V11" s="2">
+      <c r="Z11" s="1">
         <v>58</v>
       </c>
-      <c r="W11" s="2">
-        <v>64</v>
-      </c>
-      <c r="X11" s="2">
+      <c r="AA11" s="1">
+        <v>77</v>
+      </c>
+      <c r="AB11" s="2">
+        <v>46</v>
+      </c>
+      <c r="AC11" s="2">
         <v>-0.30719999999999997</v>
       </c>
-      <c r="Y11" s="1">
+      <c r="AD11" s="2">
         <v>0.2203</v>
       </c>
-      <c r="Z11" s="1">
+      <c r="AE11" s="2">
         <v>0.33339999999999997</v>
       </c>
-      <c r="AA11" s="1">
-        <v>0</v>
-      </c>
-      <c r="AB11" s="2">
+      <c r="AF11" s="1">
+        <v>-1.1496</v>
+      </c>
+      <c r="AG11" s="1">
+        <v>-0.27379999999999999</v>
+      </c>
+      <c r="AH11" s="2">
         <v>0.15</v>
       </c>
-      <c r="AC11" s="2">
+      <c r="AI11" s="2">
         <v>0.24</v>
       </c>
-      <c r="AD11" s="2">
+      <c r="AJ11" s="2">
         <v>0.24</v>
       </c>
-      <c r="AE11" s="2">
-        <v>0.24</v>
+      <c r="AK11" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="AL11" s="2">
+        <v>0.1</v>
       </c>
     </row>
-    <row r="12" spans="1:31" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:38" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>22</v>
       </c>
@@ -1555,82 +1775,103 @@
         <v>0</v>
       </c>
       <c r="G12">
-        <v>7034</v>
+        <v>7537</v>
       </c>
       <c r="H12">
+        <v>184</v>
+      </c>
+      <c r="I12">
         <v>694</v>
       </c>
-      <c r="I12">
+      <c r="J12">
         <v>261</v>
       </c>
-      <c r="J12">
-        <v>0</v>
-      </c>
       <c r="K12">
-        <v>170</v>
+        <v>0</v>
       </c>
       <c r="L12">
+        <v>1130</v>
+      </c>
+      <c r="M12">
+        <v>12</v>
+      </c>
+      <c r="N12">
         <v>22</v>
       </c>
-      <c r="M12">
+      <c r="O12">
         <v>27</v>
       </c>
-      <c r="N12">
-        <v>0</v>
-      </c>
-      <c r="O12">
-        <v>41</v>
-      </c>
       <c r="P12">
+        <v>0</v>
+      </c>
+      <c r="Q12">
+        <v>7</v>
+      </c>
+      <c r="R12">
+        <v>15</v>
+      </c>
+      <c r="S12" s="1">
         <v>679</v>
       </c>
-      <c r="Q12">
+      <c r="T12" s="1">
         <v>203</v>
       </c>
-      <c r="R12">
+      <c r="U12" s="1">
         <v>14</v>
       </c>
-      <c r="S12" s="1">
-        <v>110</v>
-      </c>
-      <c r="T12" s="1">
+      <c r="V12" s="2">
+        <v>714</v>
+      </c>
+      <c r="W12" s="2">
+        <v>6</v>
+      </c>
+      <c r="X12" s="2">
         <v>22</v>
       </c>
-      <c r="U12" s="1">
+      <c r="Y12" s="1">
         <v>35</v>
       </c>
-      <c r="V12" s="2">
-        <v>0</v>
-      </c>
-      <c r="W12" s="2">
-        <v>64</v>
-      </c>
-      <c r="X12" s="2">
+      <c r="Z12" s="1">
+        <v>0</v>
+      </c>
+      <c r="AA12" s="1">
+        <v>11</v>
+      </c>
+      <c r="AB12" s="2">
+        <v>31</v>
+      </c>
+      <c r="AC12" s="2">
         <v>-0.23219999999999999</v>
       </c>
-      <c r="Y12" s="1">
+      <c r="AD12" s="2">
         <v>-0.3982</v>
       </c>
-      <c r="Z12" s="1">
-        <v>1</v>
-      </c>
-      <c r="AA12" s="1">
-        <v>0</v>
-      </c>
-      <c r="AB12" s="2">
+      <c r="AE12" s="2">
+        <v>1</v>
+      </c>
+      <c r="AF12" s="1">
+        <v>-1.1496</v>
+      </c>
+      <c r="AG12" s="1">
+        <v>-0.27379999999999999</v>
+      </c>
+      <c r="AH12" s="2">
         <v>0.05</v>
       </c>
-      <c r="AC12" s="2">
+      <c r="AI12" s="2">
         <v>7.0000000000000007E-2</v>
       </c>
-      <c r="AD12" s="2">
+      <c r="AJ12" s="2">
         <v>0.16</v>
       </c>
-      <c r="AE12" s="2">
-        <v>0.24</v>
+      <c r="AK12" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="AL12" s="2">
+        <v>0.1</v>
       </c>
     </row>
-    <row r="13" spans="1:31" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:38" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>22</v>
       </c>
@@ -1650,82 +1891,103 @@
         <v>37212</v>
       </c>
       <c r="G13">
-        <v>12490</v>
+        <v>80942</v>
       </c>
       <c r="H13">
+        <v>4850</v>
+      </c>
+      <c r="I13">
         <v>1054</v>
       </c>
-      <c r="I13">
+      <c r="J13">
         <v>636</v>
       </c>
-      <c r="J13">
+      <c r="K13">
         <v>656</v>
       </c>
-      <c r="K13">
-        <v>197</v>
-      </c>
       <c r="L13">
+        <v>1439</v>
+      </c>
+      <c r="M13">
+        <v>122</v>
+      </c>
+      <c r="N13">
         <v>74</v>
       </c>
-      <c r="M13">
+      <c r="O13">
         <v>57</v>
       </c>
-      <c r="N13">
+      <c r="P13">
         <v>57</v>
       </c>
-      <c r="O13">
-        <v>63</v>
-      </c>
-      <c r="P13">
+      <c r="Q13">
+        <v>56</v>
+      </c>
+      <c r="R13">
+        <v>40</v>
+      </c>
+      <c r="S13" s="1">
         <v>1018</v>
       </c>
-      <c r="Q13">
+      <c r="T13" s="1">
         <v>552</v>
       </c>
-      <c r="R13">
+      <c r="U13" s="1">
         <v>558</v>
       </c>
-      <c r="S13" s="1">
-        <v>136</v>
-      </c>
-      <c r="T13" s="1">
+      <c r="V13" s="2">
+        <v>1064</v>
+      </c>
+      <c r="W13" s="2">
+        <v>69</v>
+      </c>
+      <c r="X13" s="2">
         <v>77</v>
       </c>
-      <c r="U13" s="1">
+      <c r="Y13" s="1">
         <v>65</v>
       </c>
-      <c r="V13" s="2">
+      <c r="Z13" s="1">
         <v>67</v>
       </c>
-      <c r="W13" s="2">
-        <v>92</v>
-      </c>
-      <c r="X13" s="2">
+      <c r="AA13" s="1">
+        <v>76</v>
+      </c>
+      <c r="AB13" s="2">
+        <v>70</v>
+      </c>
+      <c r="AC13" s="2">
         <v>-1.1000000000000001E-3</v>
       </c>
-      <c r="Y13" s="1">
+      <c r="AD13" s="2">
         <v>0.30359999999999998</v>
       </c>
-      <c r="Z13" s="1">
+      <c r="AE13" s="2">
         <v>0.43</v>
       </c>
-      <c r="AA13" s="1">
-        <v>0</v>
-      </c>
-      <c r="AB13" s="2">
+      <c r="AF13" s="1">
+        <v>-0.62549999999999994</v>
+      </c>
+      <c r="AG13" s="1">
+        <v>-0.50190000000000001</v>
+      </c>
+      <c r="AH13" s="2">
         <v>0.17</v>
       </c>
-      <c r="AC13" s="2">
+      <c r="AI13" s="2">
         <v>0.26</v>
       </c>
-      <c r="AD13" s="2">
+      <c r="AJ13" s="2">
         <v>0.26</v>
       </c>
-      <c r="AE13" s="2">
-        <v>0.26</v>
+      <c r="AK13" s="2">
+        <v>0.13</v>
+      </c>
+      <c r="AL13" s="2">
+        <v>0.13</v>
       </c>
     </row>
-    <row r="14" spans="1:31" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:38" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>22</v>
       </c>
@@ -1745,82 +2007,103 @@
         <v>37212</v>
       </c>
       <c r="G14">
-        <v>12490</v>
+        <v>129795</v>
       </c>
       <c r="H14">
+        <v>9980</v>
+      </c>
+      <c r="I14">
         <v>1054</v>
       </c>
-      <c r="I14">
+      <c r="J14">
         <v>636</v>
       </c>
-      <c r="J14">
+      <c r="K14">
         <v>656</v>
       </c>
-      <c r="K14">
-        <v>197</v>
-      </c>
       <c r="L14">
+        <v>1439</v>
+      </c>
+      <c r="M14">
+        <v>122</v>
+      </c>
+      <c r="N14">
         <v>74</v>
       </c>
-      <c r="M14">
+      <c r="O14">
         <v>57</v>
       </c>
-      <c r="N14">
+      <c r="P14">
         <v>57</v>
       </c>
-      <c r="O14">
-        <v>63</v>
-      </c>
-      <c r="P14">
+      <c r="Q14">
+        <v>90</v>
+      </c>
+      <c r="R14">
+        <v>82</v>
+      </c>
+      <c r="S14" s="1">
         <v>1018</v>
       </c>
-      <c r="Q14">
+      <c r="T14" s="1">
         <v>552</v>
       </c>
-      <c r="R14">
+      <c r="U14" s="1">
         <v>558</v>
       </c>
-      <c r="S14" s="1">
-        <v>136</v>
-      </c>
-      <c r="T14" s="1">
+      <c r="V14" s="2">
+        <v>1064</v>
+      </c>
+      <c r="W14" s="2">
+        <v>69</v>
+      </c>
+      <c r="X14" s="2">
         <v>77</v>
       </c>
-      <c r="U14" s="1">
+      <c r="Y14" s="1">
         <v>65</v>
       </c>
-      <c r="V14" s="2">
+      <c r="Z14" s="1">
         <v>67</v>
       </c>
-      <c r="W14" s="2">
-        <v>92</v>
-      </c>
-      <c r="X14" s="2">
+      <c r="AA14" s="1">
+        <v>122</v>
+      </c>
+      <c r="AB14" s="2">
+        <v>145</v>
+      </c>
+      <c r="AC14" s="2">
         <v>-1.1000000000000001E-3</v>
       </c>
-      <c r="Y14" s="1">
+      <c r="AD14" s="2">
         <v>0.30359999999999998</v>
       </c>
-      <c r="Z14" s="1">
+      <c r="AE14" s="2">
         <v>0.43</v>
       </c>
-      <c r="AA14" s="1">
-        <v>0</v>
-      </c>
-      <c r="AB14" s="2">
+      <c r="AF14" s="1">
+        <v>-0.62549999999999994</v>
+      </c>
+      <c r="AG14" s="1">
+        <v>-0.50190000000000001</v>
+      </c>
+      <c r="AH14" s="2">
         <v>0.17</v>
       </c>
-      <c r="AC14" s="2">
+      <c r="AI14" s="2">
         <v>0.26</v>
       </c>
-      <c r="AD14" s="2">
+      <c r="AJ14" s="2">
         <v>0.26</v>
       </c>
-      <c r="AE14" s="2">
-        <v>0.26</v>
+      <c r="AK14" s="2">
+        <v>0.13</v>
+      </c>
+      <c r="AL14" s="2">
+        <v>0.13</v>
       </c>
     </row>
-    <row r="15" spans="1:31" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:38" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>22</v>
       </c>
@@ -1840,82 +2123,103 @@
         <v>2044</v>
       </c>
       <c r="G15">
-        <v>2992</v>
+        <v>7713</v>
       </c>
       <c r="H15">
+        <v>0</v>
+      </c>
+      <c r="I15">
         <v>649</v>
       </c>
-      <c r="I15">
+      <c r="J15">
         <v>1195</v>
       </c>
-      <c r="J15">
+      <c r="K15">
         <v>92</v>
       </c>
-      <c r="K15">
-        <v>23</v>
-      </c>
       <c r="L15">
+        <v>58</v>
+      </c>
+      <c r="M15">
+        <v>0</v>
+      </c>
+      <c r="N15">
         <v>24</v>
       </c>
-      <c r="M15">
+      <c r="O15">
         <v>34</v>
       </c>
-      <c r="N15">
+      <c r="P15">
         <v>22</v>
       </c>
-      <c r="O15">
-        <v>130</v>
-      </c>
-      <c r="P15">
+      <c r="Q15">
+        <v>133</v>
+      </c>
+      <c r="R15">
+        <v>0</v>
+      </c>
+      <c r="S15" s="1">
         <v>426</v>
       </c>
-      <c r="Q15">
+      <c r="T15" s="1">
         <v>820</v>
       </c>
-      <c r="R15">
+      <c r="U15" s="1">
         <v>15</v>
       </c>
-      <c r="S15" s="1">
-        <v>24</v>
-      </c>
-      <c r="T15" s="1">
+      <c r="V15" s="2">
+        <v>54</v>
+      </c>
+      <c r="W15" s="2">
+        <v>0</v>
+      </c>
+      <c r="X15" s="2">
         <v>36</v>
       </c>
-      <c r="U15" s="1">
+      <c r="Y15" s="1">
         <v>50</v>
       </c>
-      <c r="V15" s="2">
+      <c r="Z15" s="1">
         <v>136</v>
       </c>
-      <c r="W15" s="2">
-        <v>125</v>
-      </c>
-      <c r="X15" s="2">
+      <c r="AA15" s="1">
+        <v>143</v>
+      </c>
+      <c r="AB15" s="2">
+        <v>0</v>
+      </c>
+      <c r="AC15" s="2">
         <v>0.33400000000000002</v>
       </c>
-      <c r="Y15" s="1">
+      <c r="AD15" s="2">
         <v>0.25769999999999998</v>
       </c>
-      <c r="Z15" s="1">
+      <c r="AE15" s="2">
         <v>-1.0189999999999999</v>
       </c>
-      <c r="AA15" s="1">
-        <v>0</v>
-      </c>
-      <c r="AB15" s="2">
+      <c r="AF15" s="1">
+        <v>-1.0246999999999999</v>
+      </c>
+      <c r="AG15" s="1">
+        <v>0</v>
+      </c>
+      <c r="AH15" s="2">
         <v>0.12</v>
       </c>
-      <c r="AC15" s="2">
+      <c r="AI15" s="2">
         <v>0.15</v>
       </c>
-      <c r="AD15" s="2">
+      <c r="AJ15" s="2">
         <v>0.15</v>
       </c>
-      <c r="AE15" s="2">
+      <c r="AK15" s="2">
         <v>0.17</v>
       </c>
+      <c r="AL15" s="2">
+        <v>0.17</v>
+      </c>
     </row>
-    <row r="16" spans="1:31" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:38" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>22</v>
       </c>
@@ -1926,91 +2230,112 @@
         <v>15</v>
       </c>
       <c r="D16">
-        <v>81163</v>
+        <v>124182</v>
       </c>
       <c r="E16">
-        <v>67241</v>
+        <v>147286</v>
       </c>
       <c r="F16">
-        <v>73919</v>
+        <v>162294</v>
       </c>
       <c r="G16">
-        <v>21313</v>
+        <v>194365</v>
       </c>
       <c r="H16">
-        <v>3285</v>
+        <v>12690</v>
       </c>
       <c r="I16">
-        <v>3005</v>
+        <v>5267</v>
       </c>
       <c r="J16">
-        <v>4630</v>
+        <v>5709</v>
       </c>
       <c r="K16">
-        <v>553</v>
+        <v>8091</v>
       </c>
       <c r="L16">
-        <v>25</v>
+        <v>5146</v>
       </c>
       <c r="M16">
-        <v>22</v>
+        <v>426</v>
       </c>
       <c r="N16">
-        <v>16</v>
+        <v>24</v>
       </c>
       <c r="O16">
-        <v>39</v>
+        <v>26</v>
       </c>
       <c r="P16">
-        <v>5580</v>
+        <v>20</v>
       </c>
       <c r="Q16">
-        <v>3944</v>
+        <v>38</v>
       </c>
       <c r="R16">
-        <v>4880</v>
+        <v>30</v>
       </c>
       <c r="S16" s="1">
-        <v>358</v>
+        <v>6568</v>
       </c>
       <c r="T16" s="1">
-        <v>15</v>
+        <v>5439</v>
       </c>
       <c r="U16" s="1">
-        <v>17</v>
+        <v>6683</v>
       </c>
       <c r="V16" s="2">
-        <v>15</v>
+        <v>3452</v>
       </c>
       <c r="W16" s="2">
-        <v>60</v>
+        <v>226</v>
       </c>
       <c r="X16" s="2">
-        <v>0.25180000000000002</v>
+        <v>19</v>
       </c>
       <c r="Y16" s="1">
-        <v>0.40799999999999997</v>
+        <v>27</v>
       </c>
       <c r="Z16" s="1">
-        <v>0.53249999999999997</v>
+        <v>24</v>
       </c>
       <c r="AA16" s="1">
-        <v>0</v>
+        <v>56</v>
       </c>
       <c r="AB16" s="2">
+        <v>56</v>
+      </c>
+      <c r="AC16" s="2">
+        <v>2.7400000000000001E-2</v>
+      </c>
+      <c r="AD16" s="2">
+        <v>5.9700000000000003E-2</v>
+      </c>
+      <c r="AE16" s="2">
+        <v>0.2505</v>
+      </c>
+      <c r="AF16" s="1">
+        <v>-0.1172</v>
+      </c>
+      <c r="AG16" s="1">
+        <v>-0.11409999999999999</v>
+      </c>
+      <c r="AH16" s="2">
         <v>0.05</v>
       </c>
-      <c r="AC16" s="2">
+      <c r="AI16" s="2">
         <v>0.08</v>
       </c>
-      <c r="AD16" s="2">
+      <c r="AJ16" s="2">
         <v>0.09</v>
       </c>
-      <c r="AE16" s="2">
-        <v>0.37</v>
+      <c r="AK16" s="2">
+        <v>0.14000000000000001</v>
+      </c>
+      <c r="AL16" s="2">
+        <v>0.14000000000000001</v>
       </c>
     </row>
-    <row r="17" spans="1:31" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:38" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>22</v>
       </c>
@@ -2030,82 +2355,103 @@
         <v>93552</v>
       </c>
       <c r="G17">
-        <v>21313</v>
+        <v>236554</v>
       </c>
       <c r="H17">
+        <v>24929</v>
+      </c>
+      <c r="I17">
         <v>2637</v>
       </c>
-      <c r="I17">
+      <c r="J17">
         <v>1587</v>
       </c>
-      <c r="J17">
+      <c r="K17">
         <v>1847</v>
       </c>
-      <c r="K17">
-        <v>553</v>
-      </c>
       <c r="L17">
+        <v>5146</v>
+      </c>
+      <c r="M17">
+        <v>426</v>
+      </c>
+      <c r="N17">
         <v>73</v>
       </c>
-      <c r="M17">
+      <c r="O17">
         <v>53</v>
       </c>
-      <c r="N17">
+      <c r="P17">
         <v>51</v>
       </c>
-      <c r="O17">
-        <v>39</v>
-      </c>
-      <c r="P17">
+      <c r="Q17">
+        <v>46</v>
+      </c>
+      <c r="R17">
+        <v>59</v>
+      </c>
+      <c r="S17" s="1">
         <v>1998</v>
       </c>
-      <c r="Q17">
+      <c r="T17" s="1">
         <v>1119</v>
       </c>
-      <c r="R17">
+      <c r="U17" s="1">
         <v>1073</v>
       </c>
-      <c r="S17" s="1">
-        <v>358</v>
-      </c>
-      <c r="T17" s="1">
+      <c r="V17" s="2">
+        <v>3452</v>
+      </c>
+      <c r="W17" s="2">
+        <v>226</v>
+      </c>
+      <c r="X17" s="2">
         <v>96</v>
       </c>
-      <c r="U17" s="1">
+      <c r="Y17" s="1">
         <v>76</v>
       </c>
-      <c r="V17" s="2">
+      <c r="Z17" s="1">
         <v>87</v>
       </c>
-      <c r="W17" s="2">
-        <v>60</v>
-      </c>
-      <c r="X17" s="2">
+      <c r="AA17" s="1">
+        <v>69</v>
+      </c>
+      <c r="AB17" s="2">
+        <v>110</v>
+      </c>
+      <c r="AC17" s="2">
         <v>-0.92610000000000003</v>
       </c>
-      <c r="Y17" s="1">
+      <c r="AD17" s="2">
         <v>0.43090000000000001</v>
       </c>
-      <c r="Z17" s="1">
+      <c r="AE17" s="2">
         <v>0.34539999999999998</v>
       </c>
-      <c r="AA17" s="1">
-        <v>0</v>
-      </c>
-      <c r="AB17" s="2">
+      <c r="AF17" s="1">
+        <v>-0.1172</v>
+      </c>
+      <c r="AG17" s="1">
+        <v>-0.11409999999999999</v>
+      </c>
+      <c r="AH17" s="2">
         <v>0.14000000000000001</v>
       </c>
-      <c r="AC17" s="2">
+      <c r="AI17" s="2">
         <v>0.37</v>
       </c>
-      <c r="AD17" s="2">
+      <c r="AJ17" s="2">
         <v>0.37</v>
       </c>
-      <c r="AE17" s="2">
-        <v>0.37</v>
+      <c r="AK17" s="2">
+        <v>0.14000000000000001</v>
+      </c>
+      <c r="AL17" s="2">
+        <v>0.14000000000000001</v>
       </c>
     </row>
-    <row r="18" spans="1:31" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:38" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>22</v>
       </c>
@@ -2116,91 +2462,112 @@
         <v>21</v>
       </c>
       <c r="D18">
-        <v>43018</v>
+        <v>0</v>
       </c>
       <c r="E18">
-        <v>80045</v>
+        <v>0</v>
       </c>
       <c r="F18">
-        <v>88375</v>
+        <v>0</v>
       </c>
       <c r="G18">
         <v>0</v>
       </c>
       <c r="H18">
-        <v>1982</v>
+        <v>0</v>
       </c>
       <c r="I18">
-        <v>2704</v>
+        <v>0</v>
       </c>
       <c r="J18">
-        <v>3462</v>
+        <v>0</v>
       </c>
       <c r="K18">
         <v>0</v>
       </c>
       <c r="L18">
-        <v>22</v>
+        <v>0</v>
       </c>
       <c r="M18">
-        <v>30</v>
+        <v>0</v>
       </c>
       <c r="N18">
-        <v>26</v>
+        <v>0</v>
       </c>
       <c r="O18">
         <v>0</v>
       </c>
       <c r="P18">
-        <v>988</v>
+        <v>0</v>
       </c>
       <c r="Q18">
-        <v>1495</v>
+        <v>0</v>
       </c>
       <c r="R18">
-        <v>1803</v>
+        <v>0</v>
       </c>
       <c r="S18" s="1">
         <v>0</v>
       </c>
       <c r="T18" s="1">
-        <v>44</v>
+        <v>0</v>
       </c>
       <c r="U18" s="1">
-        <v>54</v>
+        <v>0</v>
       </c>
       <c r="V18" s="2">
-        <v>49</v>
+        <v>0</v>
       </c>
       <c r="W18" s="2">
         <v>0</v>
       </c>
       <c r="X18" s="2">
-        <v>-1.2398</v>
+        <v>0</v>
       </c>
       <c r="Y18" s="1">
-        <v>-0.85909999999999997</v>
+        <v>0</v>
       </c>
       <c r="Z18" s="1">
-        <v>-0.51280000000000003</v>
+        <v>0</v>
       </c>
       <c r="AA18" s="1">
         <v>0</v>
       </c>
       <c r="AB18" s="2">
+        <v>0</v>
+      </c>
+      <c r="AC18" s="2">
+        <v>0</v>
+      </c>
+      <c r="AD18" s="2">
+        <v>0</v>
+      </c>
+      <c r="AE18" s="2">
+        <v>0</v>
+      </c>
+      <c r="AF18" s="1">
+        <v>0</v>
+      </c>
+      <c r="AG18" s="1">
+        <v>0</v>
+      </c>
+      <c r="AH18" s="2">
         <v>0.05</v>
       </c>
-      <c r="AC18" s="2">
+      <c r="AI18" s="2">
         <v>0.08</v>
       </c>
-      <c r="AD18" s="2">
+      <c r="AJ18" s="2">
         <v>0.09</v>
       </c>
-      <c r="AE18" s="2">
+      <c r="AK18" s="2">
         <v>0.37</v>
       </c>
+      <c r="AL18" s="2">
+        <v>0.37</v>
+      </c>
     </row>
-    <row r="19" spans="1:31" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:38" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>22</v>
       </c>
@@ -2220,82 +2587,103 @@
         <v>21371</v>
       </c>
       <c r="G19">
-        <v>13271</v>
+        <v>109579</v>
       </c>
       <c r="H19">
+        <v>5666</v>
+      </c>
+      <c r="I19">
         <v>623</v>
       </c>
-      <c r="I19">
+      <c r="J19">
         <v>373</v>
       </c>
-      <c r="J19">
+      <c r="K19">
         <v>406</v>
       </c>
-      <c r="K19">
-        <v>255</v>
-      </c>
       <c r="L19">
+        <v>1784</v>
+      </c>
+      <c r="M19">
+        <v>131</v>
+      </c>
+      <c r="N19">
         <v>102</v>
       </c>
-      <c r="M19">
+      <c r="O19">
         <v>49</v>
       </c>
-      <c r="N19">
+      <c r="P19">
         <v>53</v>
       </c>
-      <c r="O19">
-        <v>52</v>
-      </c>
-      <c r="P19">
+      <c r="Q19">
+        <v>61</v>
+      </c>
+      <c r="R19">
+        <v>43</v>
+      </c>
+      <c r="S19" s="1">
         <v>471</v>
       </c>
-      <c r="Q19">
+      <c r="T19" s="1">
         <v>191</v>
       </c>
-      <c r="R19">
+      <c r="U19" s="1">
         <v>199</v>
       </c>
-      <c r="S19" s="1">
-        <v>121</v>
-      </c>
-      <c r="T19" s="1">
+      <c r="V19" s="2">
+        <v>1357</v>
+      </c>
+      <c r="W19" s="2">
+        <v>84</v>
+      </c>
+      <c r="X19" s="2">
         <v>134</v>
       </c>
-      <c r="U19" s="1">
+      <c r="Y19" s="1">
         <v>97</v>
       </c>
-      <c r="V19" s="2">
+      <c r="Z19" s="1">
         <v>107</v>
       </c>
-      <c r="W19" s="2">
-        <v>110</v>
-      </c>
-      <c r="X19" s="2">
+      <c r="AA19" s="1">
+        <v>81</v>
+      </c>
+      <c r="AB19" s="2">
+        <v>67</v>
+      </c>
+      <c r="AC19" s="2">
         <v>-2.5202</v>
       </c>
-      <c r="Y19" s="1">
+      <c r="AD19" s="2">
         <v>-0.2767</v>
       </c>
-      <c r="Z19" s="1">
+      <c r="AE19" s="2">
         <v>-0.42049999999999998</v>
       </c>
-      <c r="AA19" s="1">
-        <v>0</v>
-      </c>
-      <c r="AB19" s="2">
+      <c r="AF19" s="1">
+        <v>-1.4923</v>
+      </c>
+      <c r="AG19" s="1">
+        <v>-1.0818000000000001</v>
+      </c>
+      <c r="AH19" s="2">
         <v>0.11</v>
       </c>
-      <c r="AC19" s="2">
+      <c r="AI19" s="2">
         <v>0.21</v>
       </c>
-      <c r="AD19" s="2">
+      <c r="AJ19" s="2">
         <v>0.21</v>
       </c>
-      <c r="AE19" s="2">
-        <v>0.21</v>
+      <c r="AK19" s="2">
+        <v>0.09</v>
+      </c>
+      <c r="AL19" s="2">
+        <v>0.09</v>
       </c>
     </row>
-    <row r="20" spans="1:31" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:38" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
         <v>22</v>
       </c>
@@ -2315,82 +2703,103 @@
         <v>0</v>
       </c>
       <c r="G20">
-        <v>13271</v>
+        <v>0</v>
       </c>
       <c r="H20">
+        <v>0</v>
+      </c>
+      <c r="I20">
         <v>315</v>
       </c>
-      <c r="I20">
+      <c r="J20">
         <v>398</v>
       </c>
-      <c r="J20">
-        <v>0</v>
-      </c>
       <c r="K20">
-        <v>255</v>
+        <v>0</v>
       </c>
       <c r="L20">
+        <v>1784</v>
+      </c>
+      <c r="M20">
+        <v>131</v>
+      </c>
+      <c r="N20">
         <v>23</v>
       </c>
-      <c r="M20">
+      <c r="O20">
         <v>30</v>
       </c>
-      <c r="N20">
-        <v>0</v>
-      </c>
-      <c r="O20">
-        <v>52</v>
-      </c>
       <c r="P20">
+        <v>0</v>
+      </c>
+      <c r="Q20">
+        <v>0</v>
+      </c>
+      <c r="R20">
+        <v>0</v>
+      </c>
+      <c r="S20" s="1">
         <v>81</v>
       </c>
-      <c r="Q20">
+      <c r="T20" s="1">
         <v>89</v>
       </c>
-      <c r="R20">
-        <v>0</v>
-      </c>
-      <c r="S20" s="1">
-        <v>121</v>
-      </c>
-      <c r="T20" s="1">
+      <c r="U20" s="1">
+        <v>0</v>
+      </c>
+      <c r="V20" s="2">
+        <v>1357</v>
+      </c>
+      <c r="W20" s="2">
+        <v>84</v>
+      </c>
+      <c r="X20" s="2">
         <v>88</v>
       </c>
-      <c r="U20" s="1">
+      <c r="Y20" s="1">
         <v>135</v>
       </c>
-      <c r="V20" s="2">
-        <v>0</v>
-      </c>
-      <c r="W20" s="2">
-        <v>110</v>
-      </c>
-      <c r="X20" s="2">
+      <c r="Z20" s="1">
+        <v>0</v>
+      </c>
+      <c r="AA20" s="1">
+        <v>0</v>
+      </c>
+      <c r="AB20" s="2">
+        <v>0</v>
+      </c>
+      <c r="AC20" s="2">
         <v>2.1899999999999999E-2</v>
       </c>
-      <c r="Y20" s="1">
+      <c r="AD20" s="2">
         <v>-1.8952</v>
       </c>
-      <c r="Z20" s="1">
-        <v>0</v>
-      </c>
-      <c r="AA20" s="1">
-        <v>0</v>
-      </c>
-      <c r="AB20" s="2">
+      <c r="AE20" s="2">
+        <v>0</v>
+      </c>
+      <c r="AF20" s="1">
+        <v>-1.4923</v>
+      </c>
+      <c r="AG20" s="1">
+        <v>-1.0818000000000001</v>
+      </c>
+      <c r="AH20" s="2">
         <v>0.25</v>
       </c>
-      <c r="AC20" s="2">
+      <c r="AI20" s="2">
         <v>0.13</v>
       </c>
-      <c r="AD20" s="2">
-        <v>0</v>
-      </c>
-      <c r="AE20" s="2">
-        <v>0.21</v>
+      <c r="AJ20" s="2">
+        <v>0</v>
+      </c>
+      <c r="AK20" s="2">
+        <v>0.09</v>
+      </c>
+      <c r="AL20" s="2">
+        <v>0.09</v>
       </c>
     </row>
-    <row r="21" spans="1:31" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:38" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>22</v>
       </c>
@@ -2410,82 +2819,103 @@
         <v>10281</v>
       </c>
       <c r="G21">
-        <v>6824</v>
+        <v>38931</v>
       </c>
       <c r="H21">
+        <v>2368</v>
+      </c>
+      <c r="I21">
         <v>337</v>
       </c>
-      <c r="I21">
+      <c r="J21">
         <v>147</v>
       </c>
-      <c r="J21">
+      <c r="K21">
         <v>136</v>
       </c>
-      <c r="K21">
+      <c r="L21">
+        <v>517</v>
+      </c>
+      <c r="M21">
         <v>52</v>
       </c>
-      <c r="L21">
+      <c r="N21">
         <v>121</v>
       </c>
-      <c r="M21">
+      <c r="O21">
         <v>93</v>
       </c>
-      <c r="N21">
+      <c r="P21">
         <v>76</v>
       </c>
-      <c r="O21">
+      <c r="Q21">
+        <v>75</v>
+      </c>
+      <c r="R21">
+        <v>46</v>
+      </c>
+      <c r="S21" s="1">
+        <v>310</v>
+      </c>
+      <c r="T21" s="1">
+        <v>137</v>
+      </c>
+      <c r="U21" s="1">
+        <v>124</v>
+      </c>
+      <c r="V21" s="2">
+        <v>324</v>
+      </c>
+      <c r="W21" s="2">
+        <v>23</v>
+      </c>
+      <c r="X21" s="2">
         <v>131</v>
       </c>
-      <c r="P21">
-        <v>310</v>
-      </c>
-      <c r="Q21">
-        <v>137</v>
-      </c>
-      <c r="R21">
-        <v>124</v>
-      </c>
-      <c r="S21" s="1">
-        <v>21</v>
-      </c>
-      <c r="T21" s="1">
-        <v>131</v>
-      </c>
-      <c r="U21" s="1">
+      <c r="Y21" s="1">
         <v>100</v>
       </c>
-      <c r="V21" s="2">
+      <c r="Z21" s="1">
         <v>83</v>
       </c>
-      <c r="W21" s="2">
-        <v>325</v>
-      </c>
-      <c r="X21" s="2">
+      <c r="AA21" s="1">
+        <v>120</v>
+      </c>
+      <c r="AB21" s="2">
+        <v>103</v>
+      </c>
+      <c r="AC21" s="2">
         <v>-2.1949000000000001</v>
       </c>
-      <c r="Y21" s="1">
+      <c r="AD21" s="2">
         <v>-0.54549999999999998</v>
       </c>
-      <c r="Z21" s="1">
+      <c r="AE21" s="2">
         <v>-0.27950000000000003</v>
       </c>
-      <c r="AA21" s="1">
-        <v>0</v>
-      </c>
-      <c r="AB21" s="2">
+      <c r="AF21" s="1">
+        <v>-2.3376999999999999</v>
+      </c>
+      <c r="AG21" s="1">
+        <v>-1.8597999999999999</v>
+      </c>
+      <c r="AH21" s="2">
         <v>0.11</v>
       </c>
-      <c r="AC21" s="2">
+      <c r="AI21" s="2">
         <v>0.18</v>
       </c>
-      <c r="AD21" s="2">
+      <c r="AJ21" s="2">
         <v>0.18</v>
       </c>
-      <c r="AE21" s="2">
-        <v>0.18</v>
+      <c r="AK21" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="AL21" s="2">
+        <v>0.1</v>
       </c>
     </row>
-    <row r="22" spans="1:31" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:38" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
         <v>22</v>
       </c>
@@ -2505,82 +2935,103 @@
         <v>192991</v>
       </c>
       <c r="G22">
-        <v>0</v>
+        <v>152152</v>
       </c>
       <c r="H22">
+        <v>14629</v>
+      </c>
+      <c r="I22">
         <v>1723</v>
       </c>
-      <c r="I22">
+      <c r="J22">
         <v>1935</v>
       </c>
-      <c r="J22">
+      <c r="K22">
         <v>2303</v>
       </c>
-      <c r="K22">
-        <v>0</v>
-      </c>
       <c r="L22">
+        <v>0</v>
+      </c>
+      <c r="M22">
+        <v>0</v>
+      </c>
+      <c r="N22">
         <v>74</v>
       </c>
-      <c r="M22">
+      <c r="O22">
         <v>88</v>
       </c>
-      <c r="N22">
+      <c r="P22">
         <v>84</v>
       </c>
-      <c r="O22">
-        <v>0</v>
-      </c>
-      <c r="P22">
+      <c r="Q22">
+        <v>0</v>
+      </c>
+      <c r="R22">
+        <v>0</v>
+      </c>
+      <c r="S22" s="1">
         <v>1340</v>
       </c>
-      <c r="Q22">
+      <c r="T22" s="1">
         <v>1505</v>
       </c>
-      <c r="R22">
+      <c r="U22" s="1">
         <v>1327</v>
       </c>
-      <c r="S22" s="1">
-        <v>0</v>
-      </c>
-      <c r="T22" s="1">
+      <c r="V22" s="2">
+        <v>0</v>
+      </c>
+      <c r="W22" s="2">
+        <v>0</v>
+      </c>
+      <c r="X22" s="2">
         <v>95</v>
       </c>
-      <c r="U22" s="1">
+      <c r="Y22" s="1">
         <v>114</v>
       </c>
-      <c r="V22" s="2">
+      <c r="Z22" s="1">
         <v>145</v>
       </c>
-      <c r="W22" s="2">
-        <v>0</v>
-      </c>
-      <c r="X22" s="2">
+      <c r="AA22" s="1">
+        <v>0</v>
+      </c>
+      <c r="AB22" s="2">
+        <v>0</v>
+      </c>
+      <c r="AC22" s="2">
         <v>-5.21E-2</v>
       </c>
-      <c r="Y22" s="1">
+      <c r="AD22" s="2">
         <v>-0.26319999999999999</v>
       </c>
-      <c r="Z22" s="1">
+      <c r="AE22" s="2">
         <v>-0.6159</v>
       </c>
-      <c r="AA22" s="1">
-        <v>0</v>
-      </c>
-      <c r="AB22" s="2">
+      <c r="AF22" s="1">
+        <v>0</v>
+      </c>
+      <c r="AG22" s="1">
+        <v>0</v>
+      </c>
+      <c r="AH22" s="2">
         <v>0.25</v>
       </c>
-      <c r="AC22" s="2">
+      <c r="AI22" s="2">
         <v>0.25</v>
       </c>
-      <c r="AD22" s="2">
+      <c r="AJ22" s="2">
         <v>0.25</v>
       </c>
-      <c r="AE22" s="2">
+      <c r="AK22" s="2">
+        <v>0</v>
+      </c>
+      <c r="AL22" s="2">
         <v>0</v>
       </c>
     </row>
-    <row r="23" spans="1:31" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:38" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
         <v>32</v>
       </c>
@@ -2600,82 +3051,103 @@
         <v>7316</v>
       </c>
       <c r="G23">
-        <v>0</v>
+        <v>8384</v>
       </c>
       <c r="H23">
         <v>0</v>
       </c>
       <c r="I23">
+        <v>0</v>
+      </c>
+      <c r="J23">
         <v>92</v>
       </c>
-      <c r="J23">
+      <c r="K23">
         <v>99</v>
       </c>
-      <c r="K23">
-        <v>0</v>
-      </c>
       <c r="L23">
-        <v>0</v>
+        <v>178</v>
       </c>
       <c r="M23">
+        <v>0</v>
+      </c>
+      <c r="N23">
+        <v>0</v>
+      </c>
+      <c r="O23">
         <v>53</v>
       </c>
-      <c r="N23">
+      <c r="P23">
         <v>74</v>
       </c>
-      <c r="O23">
-        <v>0</v>
-      </c>
-      <c r="P23">
-        <v>0</v>
-      </c>
       <c r="Q23">
+        <v>47</v>
+      </c>
+      <c r="R23">
+        <v>0</v>
+      </c>
+      <c r="S23" s="1">
+        <v>0</v>
+      </c>
+      <c r="T23" s="1">
         <v>26</v>
       </c>
-      <c r="R23">
+      <c r="U23" s="1">
         <v>43</v>
       </c>
-      <c r="S23" s="1">
-        <v>0</v>
-      </c>
-      <c r="T23" s="1">
-        <v>0</v>
-      </c>
-      <c r="U23" s="1">
+      <c r="V23" s="2">
+        <v>51</v>
+      </c>
+      <c r="W23" s="2">
+        <v>0</v>
+      </c>
+      <c r="X23" s="2">
+        <v>0</v>
+      </c>
+      <c r="Y23" s="1">
         <v>189</v>
       </c>
-      <c r="V23" s="2">
+      <c r="Z23" s="1">
         <v>170</v>
       </c>
-      <c r="W23" s="2">
-        <v>0</v>
-      </c>
-      <c r="X23" s="2">
-        <v>0</v>
-      </c>
-      <c r="Y23" s="1">
+      <c r="AA23" s="1">
+        <v>164</v>
+      </c>
+      <c r="AB23" s="2">
+        <v>0</v>
+      </c>
+      <c r="AC23" s="2">
+        <v>0</v>
+      </c>
+      <c r="AD23" s="2">
         <v>-0.2601</v>
       </c>
-      <c r="Z23" s="1">
+      <c r="AE23" s="2">
         <v>-0.1343</v>
       </c>
-      <c r="AA23" s="1">
-        <v>0</v>
-      </c>
-      <c r="AB23" s="2">
-        <v>1</v>
-      </c>
-      <c r="AC23" s="2">
-        <v>1</v>
-      </c>
-      <c r="AD23" s="2">
-        <v>1</v>
-      </c>
-      <c r="AE23" s="2">
+      <c r="AF23" s="1">
+        <v>-9.6000000000000002E-2</v>
+      </c>
+      <c r="AG23" s="1">
+        <v>0</v>
+      </c>
+      <c r="AH23" s="2">
+        <v>1</v>
+      </c>
+      <c r="AI23" s="2">
+        <v>1</v>
+      </c>
+      <c r="AJ23" s="2">
+        <v>1</v>
+      </c>
+      <c r="AK23" s="2">
+        <v>1</v>
+      </c>
+      <c r="AL23" s="2">
         <v>1</v>
       </c>
     </row>
-    <row r="24" spans="1:31" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:38" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
         <v>32</v>
       </c>
@@ -2695,82 +3167,103 @@
         <v>7316</v>
       </c>
       <c r="G24">
-        <v>0</v>
+        <v>44686</v>
       </c>
       <c r="H24">
         <v>0</v>
       </c>
       <c r="I24">
+        <v>0</v>
+      </c>
+      <c r="J24">
         <v>92</v>
       </c>
-      <c r="J24">
+      <c r="K24">
         <v>99</v>
       </c>
-      <c r="K24">
-        <v>0</v>
-      </c>
       <c r="L24">
-        <v>0</v>
+        <v>178</v>
       </c>
       <c r="M24">
+        <v>0</v>
+      </c>
+      <c r="N24">
+        <v>0</v>
+      </c>
+      <c r="O24">
         <v>53</v>
       </c>
-      <c r="N24">
+      <c r="P24">
         <v>74</v>
       </c>
-      <c r="O24">
-        <v>0</v>
-      </c>
-      <c r="P24">
-        <v>0</v>
-      </c>
       <c r="Q24">
+        <v>251</v>
+      </c>
+      <c r="R24">
+        <v>0</v>
+      </c>
+      <c r="S24" s="1">
+        <v>0</v>
+      </c>
+      <c r="T24" s="1">
         <v>26</v>
       </c>
-      <c r="R24">
+      <c r="U24" s="1">
         <v>43</v>
       </c>
-      <c r="S24" s="1">
-        <v>0</v>
-      </c>
-      <c r="T24" s="1">
-        <v>0</v>
-      </c>
-      <c r="U24" s="1">
+      <c r="V24" s="2">
+        <v>51</v>
+      </c>
+      <c r="W24" s="2">
+        <v>0</v>
+      </c>
+      <c r="X24" s="2">
+        <v>0</v>
+      </c>
+      <c r="Y24" s="1">
         <v>189</v>
       </c>
-      <c r="V24" s="2">
+      <c r="Z24" s="1">
         <v>170</v>
       </c>
-      <c r="W24" s="2">
-        <v>0</v>
-      </c>
-      <c r="X24" s="2">
-        <v>0</v>
-      </c>
-      <c r="Y24" s="1">
+      <c r="AA24" s="1">
+        <v>876</v>
+      </c>
+      <c r="AB24" s="2">
+        <v>0</v>
+      </c>
+      <c r="AC24" s="2">
+        <v>0</v>
+      </c>
+      <c r="AD24" s="2">
         <v>-0.2601</v>
       </c>
-      <c r="Z24" s="1">
+      <c r="AE24" s="2">
         <v>-0.1343</v>
       </c>
-      <c r="AA24" s="1">
-        <v>0</v>
-      </c>
-      <c r="AB24" s="2">
-        <v>1</v>
-      </c>
-      <c r="AC24" s="2">
-        <v>1</v>
-      </c>
-      <c r="AD24" s="2">
-        <v>1</v>
-      </c>
-      <c r="AE24" s="2">
+      <c r="AF24" s="1">
+        <v>-9.6000000000000002E-2</v>
+      </c>
+      <c r="AG24" s="1">
+        <v>0</v>
+      </c>
+      <c r="AH24" s="2">
+        <v>1</v>
+      </c>
+      <c r="AI24" s="2">
+        <v>1</v>
+      </c>
+      <c r="AJ24" s="2">
+        <v>1</v>
+      </c>
+      <c r="AK24" s="2">
+        <v>1</v>
+      </c>
+      <c r="AL24" s="2">
         <v>1</v>
       </c>
     </row>
-    <row r="25" spans="1:31" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:38" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
         <v>32</v>
       </c>
@@ -2793,11 +3286,11 @@
         <v>0</v>
       </c>
       <c r="H25">
+        <v>0</v>
+      </c>
+      <c r="I25">
         <v>35</v>
       </c>
-      <c r="I25">
-        <v>0</v>
-      </c>
       <c r="J25">
         <v>0</v>
       </c>
@@ -2805,67 +3298,88 @@
         <v>0</v>
       </c>
       <c r="L25">
+        <v>0</v>
+      </c>
+      <c r="M25">
+        <v>0</v>
+      </c>
+      <c r="N25">
         <v>22</v>
       </c>
-      <c r="M25">
-        <v>0</v>
-      </c>
-      <c r="N25">
-        <v>0</v>
-      </c>
       <c r="O25">
         <v>0</v>
       </c>
       <c r="P25">
+        <v>0</v>
+      </c>
+      <c r="Q25">
+        <v>0</v>
+      </c>
+      <c r="R25">
+        <v>0</v>
+      </c>
+      <c r="S25" s="1">
         <v>2</v>
       </c>
-      <c r="Q25">
-        <v>0</v>
-      </c>
-      <c r="R25">
-        <v>0</v>
-      </c>
-      <c r="S25" s="1">
-        <v>0</v>
-      </c>
       <c r="T25" s="1">
+        <v>0</v>
+      </c>
+      <c r="U25" s="1">
+        <v>0</v>
+      </c>
+      <c r="V25" s="2">
+        <v>0</v>
+      </c>
+      <c r="W25" s="2">
+        <v>0</v>
+      </c>
+      <c r="X25" s="2">
         <v>378</v>
       </c>
-      <c r="U25" s="1">
-        <v>0</v>
-      </c>
-      <c r="V25" s="2">
-        <v>0</v>
-      </c>
-      <c r="W25" s="2">
-        <v>0</v>
-      </c>
-      <c r="X25" s="2">
+      <c r="Y25" s="1">
+        <v>0</v>
+      </c>
+      <c r="Z25" s="1">
+        <v>0</v>
+      </c>
+      <c r="AA25" s="1">
+        <v>0</v>
+      </c>
+      <c r="AB25" s="2">
+        <v>0</v>
+      </c>
+      <c r="AC25" s="2">
         <v>-1.5216000000000001</v>
       </c>
-      <c r="Y25" s="1">
-        <v>0</v>
-      </c>
-      <c r="Z25" s="1">
-        <v>0</v>
-      </c>
-      <c r="AA25" s="1">
-        <v>0</v>
-      </c>
-      <c r="AB25" s="2">
-        <v>1</v>
-      </c>
-      <c r="AC25" s="2">
-        <v>1</v>
-      </c>
       <c r="AD25" s="2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AE25" s="2">
+        <v>0</v>
+      </c>
+      <c r="AF25" s="1">
+        <v>0</v>
+      </c>
+      <c r="AG25" s="1">
+        <v>0</v>
+      </c>
+      <c r="AH25" s="2">
+        <v>1</v>
+      </c>
+      <c r="AI25" s="2">
+        <v>1</v>
+      </c>
+      <c r="AJ25" s="2">
+        <v>1</v>
+      </c>
+      <c r="AK25" s="2">
+        <v>1</v>
+      </c>
+      <c r="AL25" s="2">
         <v>1</v>
       </c>
     </row>
-    <row r="26" spans="1:31" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:38" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
         <v>32</v>
       </c>
@@ -2948,19 +3462,40 @@
         <v>0</v>
       </c>
       <c r="AB26" s="2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AC26" s="2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AD26" s="2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AE26" s="2">
+        <v>0</v>
+      </c>
+      <c r="AF26" s="1">
+        <v>0</v>
+      </c>
+      <c r="AG26" s="1">
+        <v>0</v>
+      </c>
+      <c r="AH26" s="2">
+        <v>1</v>
+      </c>
+      <c r="AI26" s="2">
+        <v>1</v>
+      </c>
+      <c r="AJ26" s="2">
+        <v>1</v>
+      </c>
+      <c r="AK26" s="2">
         <v>0.25</v>
       </c>
+      <c r="AL26" s="2">
+        <v>0.25</v>
+      </c>
     </row>
-    <row r="27" spans="1:31" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:38" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
         <v>36</v>
       </c>
@@ -2986,10 +3521,10 @@
         <v>0</v>
       </c>
       <c r="I27">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J27">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K27">
         <v>0</v>
@@ -2998,14 +3533,14 @@
         <v>0</v>
       </c>
       <c r="M27">
+        <v>0</v>
+      </c>
+      <c r="N27">
+        <v>0</v>
+      </c>
+      <c r="O27">
         <v>418</v>
       </c>
-      <c r="N27">
-        <v>0</v>
-      </c>
-      <c r="O27">
-        <v>0</v>
-      </c>
       <c r="P27">
         <v>0</v>
       </c>
@@ -3043,19 +3578,40 @@
         <v>0</v>
       </c>
       <c r="AB27" s="2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AC27" s="2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AD27" s="2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AE27" s="2">
+        <v>0</v>
+      </c>
+      <c r="AF27" s="1">
+        <v>0</v>
+      </c>
+      <c r="AG27" s="1">
+        <v>0</v>
+      </c>
+      <c r="AH27" s="2">
+        <v>1</v>
+      </c>
+      <c r="AI27" s="2">
+        <v>1</v>
+      </c>
+      <c r="AJ27" s="2">
+        <v>1</v>
+      </c>
+      <c r="AK27" s="2">
+        <v>1</v>
+      </c>
+      <c r="AL27" s="2">
         <v>1</v>
       </c>
     </row>
-    <row r="28" spans="1:31" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:38" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
         <v>36</v>
       </c>
@@ -3081,11 +3637,11 @@
         <v>0</v>
       </c>
       <c r="I28">
+        <v>0</v>
+      </c>
+      <c r="J28">
         <v>5</v>
       </c>
-      <c r="J28">
-        <v>0</v>
-      </c>
       <c r="K28">
         <v>0</v>
       </c>
@@ -3093,14 +3649,14 @@
         <v>0</v>
       </c>
       <c r="M28">
+        <v>0</v>
+      </c>
+      <c r="N28">
+        <v>0</v>
+      </c>
+      <c r="O28">
         <v>50</v>
       </c>
-      <c r="N28">
-        <v>0</v>
-      </c>
-      <c r="O28">
-        <v>0</v>
-      </c>
       <c r="P28">
         <v>0</v>
       </c>
@@ -3138,19 +3694,40 @@
         <v>0</v>
       </c>
       <c r="AB28" s="2">
+        <v>0</v>
+      </c>
+      <c r="AC28" s="2">
+        <v>0</v>
+      </c>
+      <c r="AD28" s="2">
+        <v>0</v>
+      </c>
+      <c r="AE28" s="2">
+        <v>0</v>
+      </c>
+      <c r="AF28" s="1">
+        <v>0</v>
+      </c>
+      <c r="AG28" s="1">
+        <v>0</v>
+      </c>
+      <c r="AH28" s="2">
         <v>0.6</v>
       </c>
-      <c r="AC28" s="2">
+      <c r="AI28" s="2">
         <v>0.6</v>
       </c>
-      <c r="AD28" s="2">
+      <c r="AJ28" s="2">
         <v>0.6</v>
       </c>
-      <c r="AE28" s="2">
+      <c r="AK28" s="2">
+        <v>1</v>
+      </c>
+      <c r="AL28" s="2">
         <v>1</v>
       </c>
     </row>
-    <row r="29" spans="1:31" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:38" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
         <v>36</v>
       </c>
@@ -3244,8 +3821,29 @@
       <c r="AE29" s="2">
         <v>0</v>
       </c>
+      <c r="AF29" s="1">
+        <v>0</v>
+      </c>
+      <c r="AG29" s="1">
+        <v>0</v>
+      </c>
+      <c r="AH29" s="2">
+        <v>0</v>
+      </c>
+      <c r="AI29" s="2">
+        <v>0</v>
+      </c>
+      <c r="AJ29" s="2">
+        <v>0</v>
+      </c>
+      <c r="AK29" s="2">
+        <v>0</v>
+      </c>
+      <c r="AL29" s="2">
+        <v>0</v>
+      </c>
     </row>
-    <row r="30" spans="1:31" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:38" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
         <v>36</v>
       </c>
@@ -3271,84 +3869,105 @@
         <v>0</v>
       </c>
       <c r="I30">
+        <v>0</v>
+      </c>
+      <c r="J30">
         <v>477</v>
       </c>
-      <c r="J30">
+      <c r="K30">
         <v>65</v>
       </c>
-      <c r="K30">
-        <v>0</v>
-      </c>
       <c r="L30">
         <v>0</v>
       </c>
       <c r="M30">
+        <v>0</v>
+      </c>
+      <c r="N30">
+        <v>0</v>
+      </c>
+      <c r="O30">
         <v>43</v>
       </c>
-      <c r="N30">
+      <c r="P30">
         <v>43</v>
       </c>
-      <c r="O30">
-        <v>0</v>
-      </c>
-      <c r="P30">
-        <v>0</v>
-      </c>
       <c r="Q30">
+        <v>0</v>
+      </c>
+      <c r="R30">
+        <v>0</v>
+      </c>
+      <c r="S30">
+        <v>0</v>
+      </c>
+      <c r="T30">
         <v>200</v>
       </c>
-      <c r="R30">
+      <c r="U30">
         <v>43</v>
       </c>
-      <c r="S30">
-        <v>0</v>
-      </c>
-      <c r="T30">
-        <v>0</v>
-      </c>
-      <c r="U30">
+      <c r="V30">
+        <v>0</v>
+      </c>
+      <c r="W30">
+        <v>0</v>
+      </c>
+      <c r="X30" s="1">
+        <v>0</v>
+      </c>
+      <c r="Y30" s="1">
         <v>102</v>
       </c>
-      <c r="V30">
+      <c r="Z30" s="1">
         <v>65</v>
       </c>
-      <c r="W30">
-        <v>0</v>
-      </c>
-      <c r="X30" s="1">
-        <v>0</v>
-      </c>
-      <c r="Y30" s="1">
+      <c r="AA30" s="1">
+        <v>0</v>
+      </c>
+      <c r="AB30" s="2">
+        <v>0</v>
+      </c>
+      <c r="AC30" s="2">
+        <v>0</v>
+      </c>
+      <c r="AD30" s="2">
         <v>0.28539999999999999</v>
       </c>
-      <c r="Z30" s="1">
+      <c r="AE30" s="2">
         <v>0.56679999999999997</v>
       </c>
-      <c r="AA30" s="1">
-        <v>0</v>
-      </c>
-      <c r="AB30" s="2">
+      <c r="AF30" s="1">
+        <v>0</v>
+      </c>
+      <c r="AG30" s="1">
+        <v>0</v>
+      </c>
+      <c r="AH30" s="2">
         <v>0.95</v>
       </c>
-      <c r="AC30" s="2">
+      <c r="AI30" s="2">
         <v>0.95</v>
       </c>
-      <c r="AD30" s="2">
-        <v>1</v>
-      </c>
-      <c r="AE30" s="2">
+      <c r="AJ30" s="2">
+        <v>1</v>
+      </c>
+      <c r="AK30" s="2">
+        <v>1</v>
+      </c>
+      <c r="AL30" s="2">
         <v>1</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="7">
-    <mergeCell ref="AB1:AE1"/>
-    <mergeCell ref="D1:G1"/>
-    <mergeCell ref="H1:K1"/>
-    <mergeCell ref="L1:O1"/>
-    <mergeCell ref="P1:S1"/>
-    <mergeCell ref="T1:W1"/>
-    <mergeCell ref="X1:AA1"/>
+    <mergeCell ref="AH1:AL1"/>
+    <mergeCell ref="D1:H1"/>
+    <mergeCell ref="I1:M1"/>
+    <mergeCell ref="N1:R1"/>
+    <mergeCell ref="S1:W1"/>
+    <mergeCell ref="X1:AB1"/>
+    <mergeCell ref="AC1:AG1"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>